<commit_message>
feat: new functionality parallelism
</commit_message>
<xml_diff>
--- a/testData/TestData.xlsx
+++ b/testData/TestData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Osiris Montiel\Documents\eclipse-workspace\automation-framework-nearpedia\testData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Osiris Montiel\Documents\IdeaProjects\automation-framework-front\testData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A172E46-BC5A-43B4-B244-3A112F1F8D37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3BE5AD0-2195-4005-937F-AD3002220C45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-1875" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PortalDenuncias" sheetId="2" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="55">
   <si>
     <t>ATC0001_Nueva_Denuncia</t>
   </si>
@@ -182,6 +182,15 @@
   </si>
   <si>
     <t>Price ascending</t>
+  </si>
+  <si>
+    <t>ATC03_NearpediaTest</t>
+  </si>
+  <si>
+    <t>ATC04_NearpediaTest</t>
+  </si>
+  <si>
+    <t>ATC05_NearpediaTest</t>
   </si>
 </sst>
 </file>
@@ -249,13 +258,13 @@
   </cellStyles>
   <dxfs count="4">
     <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -274,20 +283,20 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabla13" displayName="Tabla13" ref="A1:P4" totalsRowShown="0" headerRowDxfId="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabla13" displayName="Tabla13" ref="A1:P4" totalsRowShown="0" headerRowDxfId="2">
   <autoFilter ref="A1:P4" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
   <tableColumns count="16">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="TestCaseName"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Tester"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Version"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="FolioSISAP" dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="FolioSISAP" dataDxfId="1"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Descripcion"/>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Pais"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Subsidiaria"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Categoria"/>
     <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Tipo"/>
     <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="FechaInicial"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="FechaFinal" dataDxfId="1"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="FechaFinal" dataDxfId="0"/>
     <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="NombrePersona"/>
     <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="CargoPersona"/>
     <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="InternoExterno"/>
@@ -299,8 +308,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Tabla132" displayName="Tabla132" ref="A1:E3" totalsRowShown="0" headerRowDxfId="0">
-  <autoFilter ref="A1:E3" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Tabla132" displayName="Tabla132" ref="A1:E6" totalsRowShown="0" headerRowDxfId="3">
+  <autoFilter ref="A1:E6" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="TestCaseName"/>
     <tableColumn id="5" xr3:uid="{F1AC137C-52ED-4BA8-975F-2B472EF9FAAE}" name="Ejecutar"/>
@@ -866,10 +875,69 @@
       <c r="A3" t="s">
         <v>48</v>
       </c>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
+      <c r="B3" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>52</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C4" t="s">
+        <v>44</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>53</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C5" t="s">
+        <v>44</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>51</v>
+      </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C6" t="s">
+        <v>44</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>51</v>
+      </c>
       <c r="I6" s="2"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: adding full new test case sauce demo
</commit_message>
<xml_diff>
--- a/testData/TestData.xlsx
+++ b/testData/TestData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Osiris Montiel\Documents\IdeaProjects\automation-framework-front\testData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3BE5AD0-2195-4005-937F-AD3002220C45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2838EA97-CC9C-470C-B0E6-E22D20050939}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-1875" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="68">
   <si>
     <t>ATC0001_Nueva_Denuncia</t>
   </si>
@@ -172,9 +172,6 @@
     <t>SI</t>
   </si>
   <si>
-    <t>ATC02_NearpediaTest</t>
-  </si>
-  <si>
     <t>FlightFrom</t>
   </si>
   <si>
@@ -184,20 +181,62 @@
     <t>Price ascending</t>
   </si>
   <si>
-    <t>ATC03_NearpediaTest</t>
-  </si>
-  <si>
-    <t>ATC04_NearpediaTest</t>
-  </si>
-  <si>
-    <t>ATC05_NearpediaTest</t>
+    <t>ATC02_SauceDemoTest</t>
+  </si>
+  <si>
+    <t>ATC03_SauceDemoTest</t>
+  </si>
+  <si>
+    <t>ATC04_SauceDemoTest</t>
+  </si>
+  <si>
+    <t>Username</t>
+  </si>
+  <si>
+    <t>Password</t>
+  </si>
+  <si>
+    <t>FirstName</t>
+  </si>
+  <si>
+    <t>LastName</t>
+  </si>
+  <si>
+    <t>ZipCode</t>
+  </si>
+  <si>
+    <t>standard_user</t>
+  </si>
+  <si>
+    <t>secret_sauce</t>
+  </si>
+  <si>
+    <t>Osiris</t>
+  </si>
+  <si>
+    <t>Montiel</t>
+  </si>
+  <si>
+    <t>6600</t>
+  </si>
+  <si>
+    <t>6601</t>
+  </si>
+  <si>
+    <t>6602</t>
+  </si>
+  <si>
+    <t>6603</t>
+  </si>
+  <si>
+    <t>ATC01_SauceDemoTest</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -217,6 +256,12 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -308,14 +353,19 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Tabla132" displayName="Tabla132" ref="A1:E6" totalsRowShown="0" headerRowDxfId="3">
-  <autoFilter ref="A1:E6" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
-  <tableColumns count="5">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Tabla132" displayName="Tabla132" ref="A1:J6" totalsRowShown="0" headerRowDxfId="3">
+  <autoFilter ref="A1:J6" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="TestCaseName"/>
     <tableColumn id="5" xr3:uid="{F1AC137C-52ED-4BA8-975F-2B472EF9FAAE}" name="Ejecutar"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="FlightFrom"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="FlightTo"/>
     <tableColumn id="3" xr3:uid="{2E8C600E-A409-4D88-8FD4-9D0C9284F1EF}" name="SortBy"/>
+    <tableColumn id="6" xr3:uid="{9E0C045C-4FF8-4808-8AC7-C4AA9A2F7DAB}" name="Username"/>
+    <tableColumn id="7" xr3:uid="{E1705391-AB9B-424D-8C12-A4645517AA9B}" name="Password"/>
+    <tableColumn id="8" xr3:uid="{223EDBB3-331D-4F26-9454-3ED16630127B}" name="FirstName"/>
+    <tableColumn id="9" xr3:uid="{E5826135-D33F-40E4-8ED6-5402095AD0D3}" name="LastName"/>
+    <tableColumn id="10" xr3:uid="{0A1E3F36-6458-4DEF-83AF-C98CB9CABEDE}" name="ZipCode"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -828,16 +878,20 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="52.5546875" bestFit="1" customWidth="1"/>
     <col min="2" max="3" width="14.33203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12.109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="13.5546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.88671875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>3</v>
       </c>
@@ -845,16 +899,31 @@
         <v>46</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>43</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>42</v>
       </c>
@@ -868,79 +937,111 @@
         <v>45</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>48</v>
+        <v>67</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="C3" t="s">
-        <v>44</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="E3" s="3" t="s">
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" t="s">
+        <v>59</v>
+      </c>
+      <c r="G3" t="s">
+        <v>60</v>
+      </c>
+      <c r="H3" t="s">
+        <v>61</v>
+      </c>
+      <c r="I3" t="s">
+        <v>62</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
         <v>51</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>52</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="C4" t="s">
-        <v>44</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" t="s">
+        <v>59</v>
+      </c>
+      <c r="G4" t="s">
+        <v>60</v>
+      </c>
+      <c r="H4" t="s">
+        <v>61</v>
+      </c>
+      <c r="I4" t="s">
+        <v>62</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="C5" t="s">
-        <v>44</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+      <c r="F5" t="s">
+        <v>59</v>
+      </c>
+      <c r="G5" t="s">
+        <v>60</v>
+      </c>
+      <c r="H5" t="s">
+        <v>61</v>
+      </c>
+      <c r="I5" t="s">
+        <v>62</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="C6" t="s">
-        <v>44</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="I6" s="2"/>
+      <c r="D6" s="3"/>
+      <c r="E6" s="3"/>
+      <c r="F6" t="s">
+        <v>59</v>
+      </c>
+      <c r="G6" t="s">
+        <v>60</v>
+      </c>
+      <c r="H6" t="s">
+        <v>61</v>
+      </c>
+      <c r="I6" t="s">
+        <v>62</v>
+      </c>
+      <c r="J6" s="3" t="s">
+        <v>66</v>
+      </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
   <tableParts count="1">

</xml_diff>